<commit_message>
feat(F-NAR-019): ATOM-COL.POL.001-13 Le pain chaud de Victorino
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.POL.001-13.xlsx
+++ b/stories/arbres/ATOM-COL.POL.001-13.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le cacao de Victorino</t>
+          <t>Le pain chaud de Victorino</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>café du village, puis maison</t>
+          <t>trottoir, vitre floue, pains dorés, odeur de beurre, boulangerie</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorino veut la tasse de cacao derrière la vitre. Il dit bonjour, s'il te plaît, merci. La mousse laisse un point sur son nez.</t>
+          <t>Une goutte glisse sur la vitre floue. Sur le pain, un éclat de dorure brille. Victorino veut le pain chaud maintenant. Il avance trop vite, sans le mot : la dame ne tourne pas. Il refuse de foncer, dit bonjour. Merci vécu. Le sachet glisse. Sur le pain, l'éclat de dorure tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La vapeur fait un nuage sur la vitre. Un petit rond s'ouvre, puis se referme. Ça sent le cacao, tout chaud. Une cuillère tinte contre une tasse. Le store rayé claque, dehors. Tu as vu le nuage, Victorino ? Il s'ouvre. Puis il part. C'est la vapeur du cacao. Le trottoir est encore un peu mouillé. Une feuille collée brille près du pas. On essuie tes chaussures. Voilà. J'ai les joues froides. On entre. Tu restes près de moi. En ce moment, Victorino tient la manche. La cloche de la porte fait ding. L'air est chaud, comme un câlin. Le bois du comptoir est lisse. De la mousse blanche dort dans une tasse. Celle-là. Elle a de la mousse. Le cacao bien chaud. La dame essuie encore une tasse. Le torchon est à carreaux rouges. On attend un peu. Elle a les mains prises. Victorino regarde la tasse. Il avance le doigt vers la vitre. Je veux celle-là. Tu demandes, Victorino. La dame se tourne. Un peu de mousse est sur son tablier.</t>
+          <t>Une goutte glisse sur la vitre floue. Derrière, les pains dorés attendent. Ils brillent, papa. Tu les vois, à travers le verre ? Une odeur de beurre court sur le trottoir. Ça sent le beurre, maman. Oui, le long du verre. Le trottoir est mouillé, un peu froid. Mes chaussures font toc. On les entend, sous tes pieds ? Oui, papa. On reste près de la vitre ? Oui, maman. Un pain rond se tient derrière le verre. Sa peau est dorée, un peu lisse. Celui-là, maman. Sur le pain, un éclat de dorure brille. Il est jaune, papa. C'est le pain, sous la lumière. Tu le touches, Victorino ? Victorino pose un doigt sur le verre. Le verre est tiède, un peu flou. Il pique un peu. On pousse la porte ? Oui, maintenant ! En ce moment, Victorino pose la main sur la porte. La cloche fait ding, un peu fort. L'air chaud touche les joues. Ça sent le pain et le beurre. Il est chaud ici. On reste près du bois ? Oui. Une baguette se tient debout, près du bois. Elle est grande, papa. Tu la vois, à côté du pain ? Oui. La dame essuie le bois du comptoir. Le torchon reste dans ses mains. Celui-là, maintenant ! Victorino avance trop vite vers le bois. Sa voix se mélange à la cloche. Oh. La dame ne tourne pas la tête. Le pain rond reste près du bois. Le sourire de Victorino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Elle ne m'entend pas, papa. Tu la vois, Victorino ? Papa se baisse à sa hauteur. L'éclat de dorure tremble, puis tient. Les épaules de Victorino tombent un peu. La baguette attend, là. Le mien sera chaud.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La vapeur fait un nuage sur la vitre. Un petit rond s'ouvre, puis se referme. Ça sent le cacao, tout chaud. Une cuillère tinte contre une tasse. Le store rayé claque, dehors. Tu as vu le nuage, Victorino ? Il s'ouvre. Puis il part. C'est la vapeur du cacao. Le trottoir est encore un peu mouillé. Une feuille collée brille près du pas. On essuie tes chaussures. Voilà. J'ai les joues froides. On entre. Tu restes près de moi. En ce moment, Victorino tient la manche. La cloche de la porte fait ding. L'air est chaud, comme un câlin. Le bois du comptoir est lisse. De la mousse blanche dort dans une tasse. Celle-là. Elle a de la mousse. Le cacao bien chaud. La dame essuie encore une tasse. Le torchon est à carreaux rouges. On attend un peu. Elle a les mains prises. Victorino regarde la tasse. Il avance le doigt vers la vitre. Je veux celle-là. Tu demandes, Victorino. La dame se tourne. Un peu de mousse est sur son tablier.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une goutte glisse sur la vitre floue. Derrière, les pains dorés attendent. Ils brillent, papa. Tu les vois, à travers le verre ? Une odeur de beurre court sur le trottoir. Ça sent le beurre, maman. Oui, le long du verre. Le trottoir est mouillé, un peu froid. Mes chaussures font toc. On les entend, sous tes pieds ? Oui, papa. On reste près de la vitre ? Oui, maman. Un pain rond se tient derrière le verre. Sa peau est dorée, un peu lisse. Celui-là, maman. Sur le pain, un &lt;emphasis level="moderate"&gt;éclat de dorure&lt;/emphasis&gt; brille. Il est jaune, papa. C'est le pain, sous la lumière. Tu le touches, Victorino ? Victorino pose un doigt sur le verre. Le verre est tiède, un peu flou. Il pique un peu. On pousse la porte ? Oui, maintenant ! En ce moment, Victorino pose la main sur la porte. La cloche fait ding, un peu fort. L'air chaud touche les joues. Ça sent le pain et le beurre. Il est chaud ici. On reste près du bois ? Oui. Une baguette se tient debout, près du bois. Elle est grande, papa. Tu la vois, à côté du pain ? Oui. La dame essuie le bois du comptoir. Le torchon reste dans ses mains. Celui-là, maintenant ! Victorino avance trop vite vers le bois. Sa voix se mélange à la cloche. Oh. La dame ne tourne pas la tête. Le pain rond reste près du bois. Le sourire de Victorino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Elle ne m'entend pas, papa. Tu la vois, Victorino ? Papa se baisse à sa hauteur. L'éclat de dorure tremble, puis tient. Les épaules de Victorino tombent un peu. La baguette attend, là. Le mien sera chaud.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Georges va à la boulangerie. Papa tient sa main. Ça sent le pain chaud. Georges dit : &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. La dame sourit. Georges dit : un pain, s'il te plaît. La dame tend le pain. Georges dit : merci. Papa dit : bonjour. S'il te plaît. Merci. Georges répète. Le pain est chaud. Papa dit merci aussi.&lt;/slow&gt; [pause]</t>
+          <t>Une goutte glisse sur la vitre floue. Derrière, les pains dorés attendent. Ils brillent, papa. Tu les vois, à travers le verre ? Une odeur de beurre court sur le trottoir. Ça sent le beurre, maman. Oui, le long du verre. Le trottoir est mouillé, un peu froid. Mes chaussures font toc. On les entend, sous tes pieds ? Oui, papa. On reste près de la vitre ? Oui, maman. Un pain rond se tient derrière le verre. Sa peau est dorée, un peu lisse. Celui-là, maman. Sur le pain, un &lt;emphasis&gt;éclat de dorure&lt;/emphasis&gt; brille. Il est jaune, papa. C'est le pain, sous la lumière. Tu le touches, Victorino ? Victorino pose un doigt sur le verre. Le verre est tiède, un peu flou. Il pique un peu. On pousse la porte ? Oui, maintenant ! En ce moment, Victorino pose la main sur la porte. La cloche fait ding, un peu fort. L'air chaud touche les joues. Ça sent le pain et le beurre. Il est chaud ici. On reste près du bois ? Oui. Une baguette se tient debout, près du bois. Elle est grande, papa. Tu la vois, à côté du pain ? Oui. La dame essuie le bois du comptoir. Le torchon reste dans ses mains. Celui-là, maintenant ! Victorino avance trop vite vers le bois. Sa voix se mélange à la cloche. Oh. La dame ne tourne pas la tête. Le pain rond reste près du bois. Le sourire de Victorino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Elle ne m'entend pas, papa. Tu la vois, Victorino ? Papa se baisse à sa hauteur. L'éclat de dorure tremble, puis tient. Les épaules de Victorino tombent un peu. La baguette attend, là. Le mien sera chaud. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>éclat de dorure</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,50 +1324,73 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_pain_chaud_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La vapeur fait un nuage sur la vitre.
-narrateur|Un petit rond s'ouvre, puis se referme.
-narrateur|Ça sent le cacao, tout chaud.
-narrateur|Une cuillère tinte contre une tasse.
-narrateur|Le store rayé claque, dehors.
-papa|Tu as vu le nuage, Victorino ?
-enfant-m|Il s'ouvre.
-enfant-m|Puis il part.
-papa|C'est la vapeur du cacao.
-narrateur|Le trottoir est encore un peu mouillé.
-narrateur|Une feuille collée brille près du pas.
-papa|On essuie tes chaussures.
-papa|Voilà.
-enfant-m|J'ai les joues froides.
-papa|On entre.
-papa|Tu restes près de moi.
-narrateur|En ce moment, Victorino tient la manche.
-narrateur|La cloche de la porte fait ding.
-narrateur|L'air est chaud, comme un câlin.
-narrateur|Le bois du comptoir est lisse.
-narrateur|De la mousse blanche dort dans une tasse.
-enfant-m|Celle-là.
-enfant-m|Elle a de la mousse.
-papa|Le cacao bien chaud.
-narrateur|La dame essuie encore une tasse.
-narrateur|Le torchon est à carreaux rouges.
-papa|On attend un peu.
-papa|Elle a les mains prises.
-narrateur|Victorino regarde la tasse.
-narrateur|Il avance le doigt vers la vitre.
-enfant-m|Je veux celle-là.
-papa|Tu demandes, Victorino.
-narrateur|La dame se tourne.
-narrateur|Un peu de mousse est sur son tablier.</t>
+          <t>narrateur|Une goutte glisse sur la vitre floue.
+narrateur|Derrière, les pains dorés attendent.
+enfant-m|Ils brillent, papa.
+papa|Tu les vois, à travers le verre ?
+narrateur|Une odeur de beurre court sur le trottoir.
+enfant-m|Ça sent le beurre, maman.
+maman|Oui, le long du verre.
+narrateur|Le trottoir est mouillé, un peu froid.
+enfant-m|Mes chaussures font toc.
+papa|On les entend, sous tes pieds ?
+enfant-m|Oui, papa.
+maman|On reste près de la vitre ?
+enfant-m|Oui, maman.
+narrateur|Un pain rond se tient derrière le verre.
+narrateur|Sa peau est dorée, un peu lisse.
+enfant-m|Celui-là, maman.
+narrateur|Sur le pain, un éclat de dorure brille.
+enfant-m|Il est jaune, papa.
+papa|C'est le pain, sous la lumière.
+maman|Tu le touches, Victorino ?
+narrateur|Victorino pose un doigt sur le verre.
+narrateur|Le verre est tiède, un peu flou.
+enfant-m|Il pique un peu.
+papa|On pousse la porte ?
+enfant-m|Oui, maintenant !
+narrateur|En ce moment, Victorino pose la main sur la porte.
+narrateur|La cloche fait ding, un peu fort.
+narrateur|L'air chaud touche les joues.
+narrateur|Ça sent le pain et le beurre.
+enfant-m|Il est chaud ici.
+maman|On reste près du bois ?
+enfant-m|Oui.
+narrateur|Une baguette se tient debout, près du bois.
+enfant-m|Elle est grande, papa.
+papa|Tu la vois, à côté du pain ?
+enfant-m|Oui.
+narrateur|La dame essuie le bois du comptoir.
+narrateur|Le torchon reste dans ses mains.
+enfant-m|Celui-là, maintenant !
+narrateur|Victorino avance trop vite vers le bois.
+narrateur|Sa voix se mélange à la cloche.
+enfant-m|Oh.
+narrateur|La dame ne tourne pas la tête.
+narrateur|Le pain rond reste près du bois.
+narrateur|Le sourire de Victorino disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-m|Elle ne m'entend pas, papa.
+papa|Tu la vois, Victorino ?
+narrateur|Papa se baisse à sa hauteur.
+narrateur|L'éclat de dorure tremble, puis tient.
+narrateur|Les épaules de Victorino tombent un peu.
+maman|La baguette attend, là.
+enfant-m|Le mien sera chaud.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>cloche,tasse</t>
+          <t>cloche,porte,pas</t>
         </is>
       </c>
     </row>
@@ -1394,27 +1417,27 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Victorino veut le cacao. Que dit-il ?</t>
+          <t>Victorino parle à la dame. Quels mots dit-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorino veut le cacao. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorino parle à la &lt;emphasis level="moderate"&gt;dame&lt;/emphasis&gt;. Quels mots dit-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Georges parle à la dame. Quels mots dit-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorino parle à la &lt;emphasis&gt;dame&lt;/emphasis&gt;. Quels mots dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>s'il te plaît</t>
+          <t>bonjour</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>s'il te plaît | merci | bonjour | s'il te plait</t>
+          <t>bonjour | s'il te plaît | merci | bonjour merci</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1429,7 +1452,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il dit s'il te plaît. Que dit Victorino ?</t>
+          <t>Il dit bonjour. Quels mots dit Victorino ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1467,7 +1490,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1475,10 +1498,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1493,34 +1516,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>dame</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1529,13 +1556,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1545,13 +1572,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_dit_bonjour; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Victorino veut le cacao.
-narrateur|Que dit-il ?</t>
+          <t>narrateur|Victorino parle à la dame.
+narrateur|Quels mots dit-il ?</t>
         </is>
       </c>
     </row>
@@ -1578,17 +1605,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Un cacao, s'il te plaît. Avec la mousse. La dame pose la tasse. La mousse tremble un peu. Ça sent le chocolat, tout près. Merci. Merci. Tu as demandé, Victorino. Bravo. Victorino tient l'anse des deux mains. La chaleur passe dans ses doigts. Elle est chaude, papa. On souffle un peu. Il souffle. La mousse fait un petit trou. Un point sur mon nez. Oui. Un point de mousse. La cuillère tinte encore. Le store claque, dehors. On dit au revoir, maintenant. Au revoir. Au revoir. La cloche fait ding, encore. L'air froid revient sur les joues.</t>
+          <t>Victorino avance trop vite vers le bois. Le pain, maintenant ! Sa voix se mélange à la cloche. Oh. Le torchon ne bouge pas. Le sourire ne revient pas. Victorino refuse de foncer. Il recule d'un pas, près du bois. Tu veux venir près du bois ? Papa reste à sa hauteur. Victorino écoute la cloche, un instant. Par la vitre, l'éclat de dorure brille. Bonjour. Bonjour. Un pain, s'il te plaît. Celui de la vitre. Derrière le bois, une main se tend. Le papier enveloppe le pain rond. Le sachet est chaud contre la veste. Merci. Merci, Victorino. Papa a entendu toute la phrase. Le ventre de Victorino se desserre. Il est chaud, maman. Tu as les mains dessus ? Oui, maman. Le papier est un peu gras, un peu tiède. Ça sent le beurre. On sort ? Oui, maman. Victorino tient le sachet à deux mains. Le fond du sac est tiède.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Un cacao, s'il te plaît. Avec la mousse. La dame pose la tasse. La mousse tremble un peu. Ça sent le chocolat, tout près. Merci. Merci. Tu as demandé, Victorino. Bravo. Victorino tient l'anse des deux mains. La chaleur passe dans ses doigts. Elle est chaude, papa. On souffle un peu. Il souffle. La mousse fait un petit trou. Un point sur mon nez. Oui. Un point de mousse. La cuillère tinte encore. Le store claque, dehors. On dit au revoir, maintenant. Au revoir. Au revoir. La cloche fait ding, encore. L'air froid revient sur les joues.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino avance trop vite vers le bois. Le pain, maintenant ! Sa voix se mélange à la cloche. Oh. Le torchon ne bouge pas. Le sourire ne revient pas. Victorino refuse de foncer. Il recule d'un pas, près du bois. Tu veux venir près du bois ? Papa reste à sa hauteur. Victorino écoute la cloche, un instant. Par la vitre, l'éclat de dorure brille. &lt;emphasis level="moderate"&gt;Bonjour&lt;/emphasis&gt;. Bonjour. Un pain, s'il te plaît. Celui de la vitre. Derrière le bois, une main se tend. Le papier enveloppe le pain rond. Le sachet est chaud contre la veste. Merci. Merci, Victorino. Papa a entendu toute la phrase. Le ventre de Victorino se desserre. Il est chaud, maman. Tu as les mains dessus ? Oui, maman. Le papier est un peu gras, un peu tiède. Ça sent le beurre. On sort ? Oui, maman. Victorino tient le sachet à deux mains. Le fond du sac est tiède.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Georges a dit &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Il a dit s'il te plaît. Il a dit merci. Papa était là.&lt;/slow&gt; [pause]</t>
+          <t>Victorino avance trop vite vers le bois. Le pain, maintenant ! Sa voix se mélange à la cloche. Oh. Le torchon ne bouge pas. Le sourire ne revient pas. Victorino refuse de foncer. Il recule d'un pas, près du bois. Tu veux venir près du bois ? Papa reste à sa hauteur. Victorino écoute la cloche, un instant. Par la vitre, l'éclat de dorure brille. &lt;emphasis&gt;Bonjour&lt;/emphasis&gt;. Bonjour. Un pain, s'il te plaît. Celui de la vitre. Derrière le bois, une main se tend. Le papier enveloppe le pain rond. Le sachet est chaud contre la veste. Merci. Merci, Victorino. Papa a entendu toute la phrase. Le ventre de Victorino se desserre. Il est chaud, maman. Tu as les mains dessus ? Oui, maman. Le papier est un peu gras, un peu tiède. Ça sent le beurre. On sort ? Oui, maman. Victorino tient le sachet à deux mains. Le fond du sac est tiède. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1635,18 +1662,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1669,30 +1696,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>Bonjour</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1701,10 +1728,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1713,47 +1740,52 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_salue_puis_demande; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-m|Bonjour.
-papa|Bonjour.
-enfant-m|Un cacao, s'il te plaît.
-enfant-m|Avec la mousse.
-narrateur|La dame pose la tasse.
-narrateur|La mousse tremble un peu.
-narrateur|Ça sent le chocolat, tout près.
+          <t>narrateur|Victorino avance trop vite vers le bois.
+enfant-m|Le pain, maintenant !
+narrateur|Sa voix se mélange à la cloche.
+enfant-m|Oh.
+narrateur|Le torchon ne bouge pas.
+narrateur|Le sourire ne revient pas.
+narrateur|Victorino refuse de foncer.
+narrateur|Il recule d'un pas, près du bois.
+papa|Tu veux venir près du bois ?
+narrateur|Papa reste à sa hauteur.
+narrateur|Victorino écoute la cloche, un instant.
+narrateur|Par la vitre, l'éclat de dorure brille.
+enfant-m|Bonjour.
+maman|Bonjour.
+enfant-m|Un pain, s'il te plaît.
+enfant-m|Celui de la vitre.
+narrateur|Derrière le bois, une main se tend.
+narrateur|Le papier enveloppe le pain rond.
+narrateur|Le sachet est chaud contre la veste.
 enfant-m|Merci.
-papa|Merci.
-papa|Tu as demandé, Victorino.
-papa|Bravo.
-narrateur|Victorino tient l'anse des deux mains.
-narrateur|La chaleur passe dans ses doigts.
-enfant-m|Elle est chaude, papa.
-papa|On souffle un peu.
-narrateur|Il souffle.
-narrateur|La mousse fait un petit trou.
-enfant-m|Un point sur mon nez.
-papa|Oui.
-papa|Un point de mousse.
-narrateur|La cuillère tinte encore.
-narrateur|Le store claque, dehors.
-papa|On dit au revoir, maintenant.
-enfant-m|Au revoir.
-papa|Au revoir.
-narrateur|La cloche fait ding, encore.
-narrateur|L'air froid revient sur les joues.</t>
+papa|Merci, Victorino.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Victorino se desserre.
+enfant-m|Il est chaud, maman.
+maman|Tu as les mains dessus ?
+enfant-m|Oui, maman.
+narrateur|Le papier est un peu gras, un peu tiède.
+enfant-m|Ça sent le beurre.
+maman|On sort ?
+enfant-m|Oui, maman.
+narrateur|Victorino tient le sachet à deux mains.
+narrateur|Le fond du sac est tiède.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>tasse,cuillere</t>
+          <t>papier,cloche</t>
         </is>
       </c>
     </row>
@@ -1780,17 +1812,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sur le chemin, le foulard sent le cacao. Tu as encore le point ? Un peu. Il est sucré. On le laisse. La feuille n'est plus sur le pas. Le store rayé claque loin derrière. À la maison, ça sent déjà la soupe. Vous sentez le chocolat ? C'est mon foulard. J'ai bu le cacao. Tu as demandé, Victorino ? Bonjour. S'il te plaît. Merci. La mousse a fait un point. Sur le nez ? Oui, maman. Il n'est plus là. Il est dans le foulard. Le nuage de la vitre est parti. Victorino pose le foulard sur la chaise. Ça sent encore le cacao, tout bas.</t>
+          <t>Ils passent le pas de bois. La cloche fait ding. L'air du trottoir revient sur les joues. Victorino tire le sachet trop vite. Je le montre, d'un coup ! Le papier glisse entre les doigts. Le pain rond penche vers le sol. Oh. Victorino avance les mains. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Victorino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Il ramène le sachet contre sa veste. Il écoute le trottoir, un instant. Il est chaud, papa. Tu le portes jusqu'à la rue ? Oui, papa. On marche ? Oui, maman. Une goutte glisse du verre, dehors. Elle fait un trait sur la vitre floue. Comme au début. Tu la vois, sur le verre ? Oui, maman. Victorino serre le sachet contre lui. Il reste chaud. On rentre. Le trottoir est froid, un peu lisse. Je l'entends, papa.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sur le chemin, le foulard sent le cacao. Tu as encore le point ? Un peu. Il est sucré. On le laisse. La feuille n'est plus sur le pas. Le store rayé claque loin derrière. À la maison, ça sent déjà la soupe. Vous sentez le chocolat ? C'est mon foulard. J'ai bu le cacao. Tu as demandé, Victorino ? Bonjour. S'il te plaît. Merci. La mousse a fait un point. Sur le nez ? Oui, maman. Il n'est plus là. Il est dans le foulard. Le nuage de la vitre est parti. Victorino pose le foulard sur la chaise. Ça sent encore le cacao, tout bas.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils passent le pas de bois. La cloche fait ding. L'air du trottoir revient sur les joues. Victorino tire le &lt;emphasis level="moderate"&gt;sachet&lt;/emphasis&gt; trop vite. Je le montre, d'un coup ! Le papier glisse entre les doigts. Le pain rond penche vers le sol. Oh. Victorino avance les mains. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Victorino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Il ramène le sachet contre sa veste. Il écoute le trottoir, un instant. Il est chaud, papa. Tu le portes jusqu'à la rue ? Oui, papa. On marche ? Oui, maman. Une goutte glisse du verre, dehors. Elle fait un trait sur la vitre floue. Comme au début. Tu la vois, sur le verre ? Oui, maman. Victorino serre le sachet contre lui. Il reste chaud. On rentre. Le trottoir est froid, un peu lisse. Je l'entends, papa.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Georges tient le pain. Papa ouvre la porte.&lt;/slow&gt; [pause]</t>
+          <t>Ils passent le pas de bois. La cloche fait ding. L'air du trottoir revient sur les joues. Victorino tire le &lt;emphasis&gt;sachet&lt;/emphasis&gt; trop vite. Je le montre, d'un coup ! Le papier glisse entre les doigts. Le pain rond penche vers le sol. Oh. Victorino avance les mains. Puis il s'arrête net. Attends, je regarde. Papa attend, sans parler. Victorino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Il ramène le sachet contre sa veste. Il écoute le trottoir, un instant. Il est chaud, papa. Tu le portes jusqu'à la rue ? Oui, papa. On marche ? Oui, maman. Une goutte glisse du verre, dehors. Elle fait un trait sur la vitre floue. Comme au début. Tu la vois, sur le verre ? Oui, maman. Victorino serre le sachet contre lui. Il reste chaud. On rentre. Le trottoir est froid, un peu lisse. Je l'entends, papa. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1837,18 +1869,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1869,28 +1901,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>sachet</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1899,10 +1935,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1911,39 +1947,51 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_quand_le_sachet_glisse; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Sur le chemin, le foulard sent le cacao.
-papa|Tu as encore le point ?
-enfant-m|Un peu.
-enfant-m|Il est sucré.
-papa|On le laisse.
-narrateur|La feuille n'est plus sur le pas.
-narrateur|Le store rayé claque loin derrière.
-narrateur|À la maison, ça sent déjà la soupe.
-maman|Vous sentez le chocolat ?
-enfant-m|C'est mon foulard.
-enfant-m|J'ai bu le cacao.
-maman|Tu as demandé, Victorino ?
-enfant-m|Bonjour.
-enfant-m|S'il te plaît.
-enfant-m|Merci.
-papa|La mousse a fait un point.
-maman|Sur le nez ?
+          <t>narrateur|Ils passent le pas de bois.
+narrateur|La cloche fait ding.
+narrateur|L'air du trottoir revient sur les joues.
+narrateur|Victorino tire le sachet trop vite.
+enfant-m|Je le montre, d'un coup !
+narrateur|Le papier glisse entre les doigts.
+narrateur|Le pain rond penche vers le sol.
+enfant-m|Oh.
+narrateur|Victorino avance les mains.
+narrateur|Puis il s'arrête net.
+enfant-m|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Victorino refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Il ramène le sachet contre sa veste.
+narrateur|Il écoute le trottoir, un instant.
+enfant-m|Il est chaud, papa.
+papa|Tu le portes jusqu'à la rue ?
+enfant-m|Oui, papa.
+maman|On marche ?
 enfant-m|Oui, maman.
-maman|Il n'est plus là.
-enfant-m|Il est dans le foulard.
-papa|Le nuage de la vitre est parti.
-narrateur|Victorino pose le foulard sur la chaise.
-narrateur|Ça sent encore le cacao, tout bas.</t>
+narrateur|Une goutte glisse du verre, dehors.
+narrateur|Elle fait un trait sur la vitre floue.
+enfant-m|Comme au début.
+maman|Tu la vois, sur le verre ?
+enfant-m|Oui, maman.
+narrateur|Victorino serre le sachet contre lui.
+enfant-m|Il reste chaud.
+papa|On rentre.
+narrateur|Le trottoir est froid, un peu lisse.
+enfant-m|Je l'entends, papa.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>pas,porte</t>
+          <t>pas,papier</t>
         </is>
       </c>
     </row>
@@ -1970,17 +2018,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le foulard repose sur la chaise. Il sent encore le cacao. Bonne soirée, Victorino. La tasse était chaude.</t>
+          <t>Ils s'arrêtent sous la vitre floue. La goutte a fini sa course. Le pain brillait, papa. Tu le vois, comme dans la boutique ? Oui, sur le pain. Victorino pose le sachet contre la veste. On le garde au chaud ? Oui, maman. Ça sent le beurre, maman. Il est contre toi. Une vapeur monte du papier. Victorino respire, plus large. On rentre ? Oui. Les joues de Victorino se réchauffent. Le sachet reste tiède sous la main. On le voit, maman. Tu le vois sur le pain ? Oui, l'éclat. L'éclat de dorure tient sur le pain.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le foulard repose sur la chaise. Il sent encore le cacao. Bonne soirée, Victorino. La tasse était chaude.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils s'arrêtent sous la vitre floue. La goutte a fini sa course. Le pain brillait, papa. Tu le vois, comme dans la boutique ? Oui, sur le pain. Victorino pose le sachet contre la veste. On le garde au chaud ? Oui, maman. Ça sent le beurre, maman. Il est contre toi. Une vapeur monte du papier. Victorino respire, plus large. On rentre ? Oui. Les joues de Victorino se réchauffent. Le sachet reste tiède sous la main. On le voit, maman. Tu le vois sur le pain ? Oui, l'éclat. L'&lt;emphasis level="moderate"&gt;éclat de dorure&lt;/emphasis&gt; tient sur le pain.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils s'arrêtent sous la vitre floue. La goutte a fini sa course. Le pain brillait, papa. Tu le vois, comme dans la boutique ? Oui, sur le pain. Victorino pose le sachet contre la veste. On le garde au chaud ? Oui, maman. Ça sent le beurre, maman. Il est contre toi. Une vapeur monte du papier. Victorino respire, plus large. On rentre ? Oui. Les joues de Victorino se réchauffent. Le sachet reste tiède sous la main. On le voit, maman. Tu le vois sur le pain ? Oui, l'éclat. L'&lt;emphasis&gt;éclat de dorure&lt;/emphasis&gt; tient sur le pain.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2027,7 +2075,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2035,10 +2083,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2047,12 +2095,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2061,17 +2109,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de dorure</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2080,11 +2132,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2093,27 +2145,52 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_pain; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le foulard repose sur la chaise.
-narrateur|Il sent encore le cacao.
-maman|Bonne soirée, Victorino.
-papa|La tasse était chaude.</t>
+          <t>narrateur|Ils s'arrêtent sous la vitre floue.
+narrateur|La goutte a fini sa course.
+enfant-m|Le pain brillait, papa.
+papa|Tu le vois, comme dans la boutique ?
+enfant-m|Oui, sur le pain.
+narrateur|Victorino pose le sachet contre la veste.
+maman|On le garde au chaud ?
+enfant-m|Oui, maman.
+enfant-m|Ça sent le beurre, maman.
+maman|Il est contre toi.
+narrateur|Une vapeur monte du papier.
+narrateur|Victorino respire, plus large.
+papa|On rentre ?
+enfant-m|Oui.
+narrateur|Les joues de Victorino se réchauffent.
+narrateur|Le sachet reste tiède sous la main.
+enfant-m|On le voit, maman.
+maman|Tu le vois sur le pain ?
+enfant-m|Oui, l'éclat.
+narrateur|L'éclat de dorure tient sur le pain.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>pain,verre</t>
         </is>
       </c>
     </row>
@@ -2134,7 +2211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2219,6 +2296,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>